<commit_message>
Scheduled Cleaned - Complete
</commit_message>
<xml_diff>
--- a/Cleaned_Schedule/class_schedule_BSCS-4.xlsx
+++ b/Cleaned_Schedule/class_schedule_BSCS-4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neera\OneDrive\University\Spring 2025\AI\Project\Cleaned_Schedule\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7310C006-B675-4993-8001-DD4D5BC550C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6C9918C-DAD3-41A1-9C25-6396FAB8143D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="fc898cd5-f00c-4aee-b7a7-fcde217" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="77">
   <si>
     <t>Class Timing</t>
   </si>
@@ -229,21 +229,6 @@
     <t xml:space="preserve">Ms. Mewish Zafar </t>
   </si>
   <si>
-    <t>MTC-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dr.Tahir Syed </t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Computer Communication and Networking (Lab) Only Tuesday 
-11:30 am to 2:15 pm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Mr. M. Waseem Arain</t>
-  </si>
-  <si>
     <t>Dr.Tahir Syed</t>
   </si>
   <si>
@@ -253,17 +238,38 @@
     <t xml:space="preserve">8:30 am to 9:45 am </t>
   </si>
   <si>
-    <t xml:space="preserve">PENDING TUESDAY THRUDAY, still cleaning this data </t>
-  </si>
-  <si>
     <t xml:space="preserve">10:00 am to 11:15 am </t>
+  </si>
+  <si>
+    <t>Computer Communication and Networking (Lab) Only Tuesday 11:30 am to 2:15 pm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thrusday </t>
+  </si>
+  <si>
+    <t>Computer Architecture and Assembly Language (Lab) Only Friday 8:30 to 11:15 am</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ms. Asma Tauqir </t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>Pakistan History Only Saturday 8:30 to 11:15 am</t>
+  </si>
+  <si>
+    <t>MAC-3</t>
+  </si>
+  <si>
+    <t>Saturday</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -271,12 +277,6 @@
     </font>
     <font>
       <sz val="8"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -301,9 +301,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -431,14 +434,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M52"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.109375" customWidth="1"/>
-    <col min="2" max="2" width="75.44140625" customWidth="1"/>
+    <col min="2" max="2" width="88.5546875" customWidth="1"/>
     <col min="3" max="3" width="8.33203125" customWidth="1"/>
     <col min="4" max="4" width="10.21875" customWidth="1"/>
-    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="5" max="5" width="22.44140625" customWidth="1"/>
     <col min="6" max="6" width="19.21875" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
     <col min="9" max="9" width="74.21875" customWidth="1"/>
@@ -1180,7 +1183,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>42</v>
       </c>
@@ -1203,134 +1206,202 @@
         <v>47</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B38" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>67</v>
+      </c>
+      <c r="B34" t="s">
+        <v>51</v>
+      </c>
+      <c r="C34" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" t="s">
+        <v>24</v>
+      </c>
+      <c r="E34">
+        <v>98503</v>
+      </c>
+      <c r="F34" t="s">
+        <v>34</v>
+      </c>
+      <c r="G34" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>68</v>
+      </c>
+      <c r="B35" t="s">
+        <v>51</v>
+      </c>
+      <c r="C35" t="s">
+        <v>9</v>
+      </c>
+      <c r="D35" t="s">
+        <v>24</v>
+      </c>
+      <c r="E35">
+        <v>98503</v>
+      </c>
+      <c r="F35" t="s">
+        <v>34</v>
+      </c>
+      <c r="G35" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>68</v>
+      </c>
+      <c r="B36" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36" t="s">
+        <v>9</v>
+      </c>
+      <c r="D36" t="s">
+        <v>52</v>
+      </c>
+      <c r="E36">
+        <v>98464</v>
+      </c>
+      <c r="F36" t="s">
+        <v>53</v>
+      </c>
+      <c r="G36" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>68</v>
+      </c>
+      <c r="B37" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" t="s">
+        <v>9</v>
+      </c>
+      <c r="D37" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37">
+        <v>98470</v>
+      </c>
+      <c r="F37" t="s">
+        <v>29</v>
+      </c>
+      <c r="G37" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>68</v>
+      </c>
+      <c r="B38" t="s">
+        <v>18</v>
+      </c>
+      <c r="C38" t="s">
+        <v>9</v>
+      </c>
+      <c r="D38" t="s">
+        <v>54</v>
+      </c>
+      <c r="E38">
+        <v>98471</v>
+      </c>
+      <c r="F38" t="s">
+        <v>55</v>
+      </c>
+      <c r="G38" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B39" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C39" t="s">
         <v>9</v>
       </c>
       <c r="D39" t="s">
-        <v>24</v>
-      </c>
-      <c r="E39">
-        <v>98503</v>
+        <v>22</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>57</v>
       </c>
       <c r="F39" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="G39" t="s">
         <v>46</v>
       </c>
-      <c r="I39" t="s">
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>48</v>
+      </c>
+      <c r="B40" t="s">
         <v>14</v>
       </c>
-      <c r="J39" t="s">
-        <v>9</v>
-      </c>
-      <c r="K39" t="s">
-        <v>52</v>
-      </c>
-      <c r="L39">
-        <v>98464</v>
-      </c>
-      <c r="M39" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>73</v>
-      </c>
-      <c r="B40" t="s">
-        <v>51</v>
-      </c>
       <c r="C40" t="s">
         <v>9</v>
       </c>
       <c r="D40" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="E40">
-        <v>98503</v>
+        <v>98493</v>
       </c>
       <c r="F40" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="G40" t="s">
         <v>46</v>
       </c>
-      <c r="I40" t="s">
-        <v>18</v>
-      </c>
-      <c r="J40" t="s">
-        <v>9</v>
-      </c>
-      <c r="K40" t="s">
-        <v>19</v>
-      </c>
-      <c r="L40">
-        <v>98470</v>
-      </c>
-      <c r="M40" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>73</v>
+    </row>
+    <row r="41" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>48</v>
       </c>
       <c r="B41" t="s">
-        <v>14</v>
+        <v>59</v>
       </c>
       <c r="C41" t="s">
         <v>9</v>
       </c>
       <c r="D41" t="s">
-        <v>52</v>
-      </c>
-      <c r="E41">
-        <v>98464</v>
+        <v>60</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>61</v>
       </c>
       <c r="F41" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G41" t="s">
         <v>46</v>
       </c>
-      <c r="I41" t="s">
-        <v>18</v>
-      </c>
-      <c r="J41" t="s">
-        <v>9</v>
-      </c>
-      <c r="K41" t="s">
-        <v>54</v>
-      </c>
-      <c r="L41">
-        <v>98471</v>
-      </c>
-      <c r="M41" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>48</v>
+      </c>
       <c r="B42" t="s">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="C42" t="s">
         <v>9</v>
       </c>
       <c r="D42" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="E42">
         <v>98470</v>
@@ -1341,235 +1412,488 @@
       <c r="G42" t="s">
         <v>46</v>
       </c>
-      <c r="I42" t="s">
-        <v>56</v>
-      </c>
-      <c r="J42" t="s">
-        <v>9</v>
-      </c>
-      <c r="K42" t="s">
-        <v>22</v>
-      </c>
-      <c r="L42" t="s">
-        <v>57</v>
-      </c>
-      <c r="M42" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>48</v>
+      </c>
       <c r="B43" t="s">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="C43" t="s">
         <v>9</v>
       </c>
       <c r="D43" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="E43">
         <v>98471</v>
       </c>
       <c r="F43" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G43" t="s">
         <v>46</v>
       </c>
-      <c r="I43" t="s">
-        <v>51</v>
-      </c>
-      <c r="J43" t="s">
-        <v>9</v>
-      </c>
-      <c r="K43" t="s">
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>49</v>
+      </c>
+      <c r="B44" t="s">
+        <v>62</v>
+      </c>
+      <c r="C44" t="s">
+        <v>9</v>
+      </c>
+      <c r="D44" t="s">
         <v>24</v>
       </c>
-      <c r="L43">
-        <v>98503</v>
-      </c>
-      <c r="M43" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B44" t="s">
-        <v>56</v>
-      </c>
-      <c r="C44" t="s">
-        <v>9</v>
-      </c>
-      <c r="D44" t="s">
-        <v>22</v>
-      </c>
-      <c r="E44" t="s">
-        <v>57</v>
+      <c r="E44">
+        <v>98470</v>
       </c>
       <c r="F44" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="G44" t="s">
         <v>46</v>
       </c>
-      <c r="I44" t="s">
-        <v>14</v>
-      </c>
-      <c r="J44" t="s">
-        <v>9</v>
-      </c>
-      <c r="K44" t="s">
-        <v>15</v>
-      </c>
-      <c r="L44">
-        <v>98493</v>
-      </c>
-      <c r="M44" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>49</v>
+      </c>
+      <c r="B45" t="s">
+        <v>62</v>
+      </c>
+      <c r="C45" t="s">
+        <v>9</v>
+      </c>
+      <c r="D45" t="s">
+        <v>24</v>
+      </c>
+      <c r="E45">
+        <v>98471</v>
+      </c>
+      <c r="F45" t="s">
+        <v>25</v>
+      </c>
       <c r="G45" t="s">
         <v>46</v>
       </c>
-      <c r="I45" t="s">
-        <v>59</v>
-      </c>
-      <c r="J45" t="s">
-        <v>9</v>
-      </c>
-      <c r="K45" t="s">
-        <v>60</v>
-      </c>
-      <c r="L45" t="s">
-        <v>61</v>
-      </c>
-      <c r="M45" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>49</v>
+      </c>
+      <c r="B46" t="s">
+        <v>63</v>
+      </c>
+      <c r="C46" t="s">
+        <v>9</v>
+      </c>
+      <c r="D46" t="s">
+        <v>27</v>
+      </c>
+      <c r="E46">
+        <v>98496</v>
+      </c>
+      <c r="F46" t="s">
+        <v>64</v>
+      </c>
       <c r="G46" t="s">
         <v>46</v>
       </c>
-      <c r="I46" t="s">
-        <v>62</v>
-      </c>
-      <c r="J46" t="s">
-        <v>9</v>
-      </c>
-      <c r="K46" t="s">
-        <v>24</v>
-      </c>
-      <c r="L46">
-        <v>98470</v>
-      </c>
-      <c r="M46" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" t="s">
+        <v>14</v>
+      </c>
+      <c r="C47" t="s">
+        <v>9</v>
+      </c>
+      <c r="D47" t="s">
+        <v>15</v>
+      </c>
+      <c r="E47">
+        <v>98505</v>
+      </c>
+      <c r="F47" t="s">
+        <v>65</v>
+      </c>
       <c r="G47" t="s">
         <v>46</v>
       </c>
-      <c r="I47" t="s">
-        <v>63</v>
-      </c>
-      <c r="J47" t="s">
-        <v>9</v>
-      </c>
-      <c r="K47" t="s">
-        <v>27</v>
-      </c>
-      <c r="L47">
-        <v>98496</v>
-      </c>
-      <c r="M47" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>37</v>
+      </c>
+      <c r="B48" t="s">
+        <v>14</v>
+      </c>
+      <c r="C48" t="s">
+        <v>9</v>
+      </c>
+      <c r="D48" t="s">
+        <v>15</v>
+      </c>
+      <c r="E48">
+        <v>98512</v>
+      </c>
+      <c r="F48" t="s">
+        <v>65</v>
+      </c>
       <c r="G48" t="s">
         <v>46</v>
       </c>
-      <c r="I48" t="s">
-        <v>14</v>
-      </c>
-      <c r="J48" t="s">
-        <v>9</v>
-      </c>
-      <c r="K48" t="s">
-        <v>65</v>
-      </c>
-      <c r="L48">
-        <v>98505</v>
-      </c>
-      <c r="M48" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="49" spans="7:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>37</v>
+      </c>
+      <c r="B49" t="s">
+        <v>63</v>
+      </c>
+      <c r="C49" t="s">
+        <v>9</v>
+      </c>
+      <c r="D49" t="s">
+        <v>27</v>
+      </c>
+      <c r="E49">
+        <v>98496</v>
+      </c>
+      <c r="F49" t="s">
+        <v>64</v>
+      </c>
       <c r="G49" t="s">
         <v>46</v>
       </c>
-      <c r="I49" t="s">
-        <v>67</v>
-      </c>
-      <c r="J49" t="s">
-        <v>9</v>
-      </c>
-      <c r="K49" t="s">
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>37</v>
+      </c>
+      <c r="B50" t="s">
+        <v>66</v>
+      </c>
+      <c r="C50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D50" t="s">
         <v>24</v>
       </c>
-      <c r="L49">
-        <v>98470</v>
-      </c>
-      <c r="M49" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="50" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="E50">
+        <v>98473</v>
+      </c>
+      <c r="F50" t="s">
+        <v>58</v>
+      </c>
       <c r="G50" t="s">
         <v>46</v>
       </c>
-      <c r="I50" t="s">
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>68</v>
+      </c>
+      <c r="B51" t="s">
         <v>14</v>
       </c>
-      <c r="J50" t="s">
-        <v>9</v>
-      </c>
-      <c r="K50" t="s">
+      <c r="C51" t="s">
+        <v>9</v>
+      </c>
+      <c r="D51" t="s">
+        <v>52</v>
+      </c>
+      <c r="E51">
+        <v>98464</v>
+      </c>
+      <c r="F51" t="s">
+        <v>53</v>
+      </c>
+      <c r="G51" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>68</v>
+      </c>
+      <c r="B52" t="s">
+        <v>18</v>
+      </c>
+      <c r="C52" t="s">
+        <v>9</v>
+      </c>
+      <c r="D52" t="s">
+        <v>19</v>
+      </c>
+      <c r="E52">
+        <v>98470</v>
+      </c>
+      <c r="F52" t="s">
+        <v>29</v>
+      </c>
+      <c r="G52" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>68</v>
+      </c>
+      <c r="B53" t="s">
+        <v>18</v>
+      </c>
+      <c r="C53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D53" t="s">
+        <v>54</v>
+      </c>
+      <c r="E53">
+        <v>98471</v>
+      </c>
+      <c r="F53" t="s">
+        <v>55</v>
+      </c>
+      <c r="G53" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>68</v>
+      </c>
+      <c r="B54" t="s">
+        <v>56</v>
+      </c>
+      <c r="C54" t="s">
+        <v>9</v>
+      </c>
+      <c r="D54" t="s">
+        <v>22</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F54" t="s">
+        <v>58</v>
+      </c>
+      <c r="G54" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>48</v>
+      </c>
+      <c r="B55" t="s">
+        <v>14</v>
+      </c>
+      <c r="C55" t="s">
+        <v>9</v>
+      </c>
+      <c r="D55" t="s">
         <v>15</v>
       </c>
-      <c r="L50">
+      <c r="E55">
+        <v>98493</v>
+      </c>
+      <c r="F55" t="s">
+        <v>16</v>
+      </c>
+      <c r="G55" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B56" t="s">
+        <v>59</v>
+      </c>
+      <c r="C56" t="s">
+        <v>9</v>
+      </c>
+      <c r="D56" t="s">
+        <v>60</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F56" t="s">
+        <v>58</v>
+      </c>
+      <c r="G56" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>37</v>
+      </c>
+      <c r="B57" t="s">
+        <v>14</v>
+      </c>
+      <c r="C57" t="s">
+        <v>9</v>
+      </c>
+      <c r="D57" t="s">
+        <v>15</v>
+      </c>
+      <c r="E57">
         <v>98512</v>
       </c>
-      <c r="M50" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="51" spans="7:13" x14ac:dyDescent="0.25">
-      <c r="G51" t="s">
-        <v>46</v>
-      </c>
-      <c r="I51" t="s">
+      <c r="F57" t="s">
+        <v>65</v>
+      </c>
+      <c r="G57" t="s">
         <v>70</v>
       </c>
-      <c r="J51" t="s">
-        <v>9</v>
-      </c>
-      <c r="K51" t="s">
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>37</v>
+      </c>
+      <c r="B58" t="s">
+        <v>63</v>
+      </c>
+      <c r="C58" t="s">
+        <v>9</v>
+      </c>
+      <c r="D58" t="s">
+        <v>27</v>
+      </c>
+      <c r="E58">
+        <v>98496</v>
+      </c>
+      <c r="F58" t="s">
+        <v>64</v>
+      </c>
+      <c r="G58" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>37</v>
+      </c>
+      <c r="B59" t="s">
+        <v>66</v>
+      </c>
+      <c r="C59" t="s">
+        <v>9</v>
+      </c>
+      <c r="D59" t="s">
         <v>24</v>
       </c>
-      <c r="L51">
+      <c r="E59">
         <v>98473</v>
       </c>
-      <c r="M51" t="s">
+      <c r="F59" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="52" spans="7:13" x14ac:dyDescent="0.25">
-      <c r="G52" t="s">
-        <v>46</v>
+      <c r="G59" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>7</v>
+      </c>
+      <c r="B60" t="s">
+        <v>71</v>
+      </c>
+      <c r="C60" t="s">
+        <v>9</v>
+      </c>
+      <c r="D60" t="s">
+        <v>33</v>
+      </c>
+      <c r="E60">
+        <v>98473</v>
+      </c>
+      <c r="F60" t="s">
+        <v>72</v>
+      </c>
+      <c r="G60" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>68</v>
+      </c>
+      <c r="B61" t="s">
+        <v>71</v>
+      </c>
+      <c r="C61" t="s">
+        <v>9</v>
+      </c>
+      <c r="D61" t="s">
+        <v>33</v>
+      </c>
+      <c r="E61">
+        <v>98473</v>
+      </c>
+      <c r="F61" t="s">
+        <v>72</v>
+      </c>
+      <c r="G61" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>7</v>
+      </c>
+      <c r="B62" t="s">
+        <v>74</v>
+      </c>
+      <c r="C62" t="s">
+        <v>9</v>
+      </c>
+      <c r="D62" t="s">
+        <v>75</v>
+      </c>
+      <c r="E62">
+        <v>98525</v>
+      </c>
+      <c r="F62" t="s">
+        <v>13</v>
+      </c>
+      <c r="G62" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>17</v>
+      </c>
+      <c r="B63" t="s">
+        <v>74</v>
+      </c>
+      <c r="C63" t="s">
+        <v>9</v>
+      </c>
+      <c r="D63" t="s">
+        <v>75</v>
+      </c>
+      <c r="E63">
+        <v>98525</v>
+      </c>
+      <c r="F63" t="s">
+        <v>13</v>
+      </c>
+      <c r="G63" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Comments in Schedule
</commit_message>
<xml_diff>
--- a/Cleaned_Schedule/class_schedule_BSCS-4.xlsx
+++ b/Cleaned_Schedule/class_schedule_BSCS-4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neera\OneDrive\University\Spring 2025\AI\Project\Cleaned_Schedule\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6C9918C-DAD3-41A1-9C25-6396FAB8143D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{652DE80D-BC8D-40DC-B111-3785A2818E5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="fc898cd5-f00c-4aee-b7a7-fcde217" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="84">
   <si>
     <t>Class Timing</t>
   </si>
@@ -200,10 +200,6 @@
     <t xml:space="preserve">Computer Architecture and Assembly Language (2 Merge Sessions) </t>
   </si>
   <si>
-    <t>98472
-98496</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dr. Salman Zafar </t>
   </si>
   <si>
@@ -211,10 +207,6 @@
   </si>
   <si>
     <t>MTS 7</t>
-  </si>
-  <si>
-    <t>98503
-98504</t>
   </si>
   <si>
     <t xml:space="preserve">Computer Communication and Networking (Lab) Only Tuesday 
@@ -263,6 +255,33 @@
   </si>
   <si>
     <t>Saturday</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comments </t>
+  </si>
+  <si>
+    <t>Lecture</t>
+  </si>
+  <si>
+    <t>2 Combined Sessions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lab Only Monday </t>
+  </si>
+  <si>
+    <t>Lab Only Monday</t>
+  </si>
+  <si>
+    <t>Lab Only Wednesday</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lab Only Tuesday </t>
+  </si>
+  <si>
+    <t>Lab Only Friday</t>
+  </si>
+  <si>
+    <t>2 Merge Sessions</t>
   </si>
 </sst>
 </file>
@@ -434,7 +453,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.109375" customWidth="1"/>
@@ -444,10 +463,11 @@
     <col min="5" max="5" width="22.44140625" customWidth="1"/>
     <col min="6" max="6" width="19.21875" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
+    <col min="8" max="8" width="27.109375" customWidth="1"/>
     <col min="9" max="9" width="74.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -469,8 +489,11 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -492,8 +515,11 @@
       <c r="G2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -515,8 +541,11 @@
       <c r="G3" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -538,8 +567,11 @@
       <c r="G4" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -561,8 +593,11 @@
       <c r="G5" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -584,8 +619,11 @@
       <c r="G6" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -607,8 +645,11 @@
       <c r="G7" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -630,8 +671,11 @@
       <c r="G8" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>48</v>
       </c>
@@ -653,8 +697,11 @@
       <c r="G9" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>48</v>
       </c>
@@ -676,8 +723,11 @@
       <c r="G10" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>49</v>
       </c>
@@ -699,8 +749,11 @@
       <c r="G11" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H11" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>49</v>
       </c>
@@ -722,8 +775,11 @@
       <c r="G12" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H12" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -745,8 +801,11 @@
       <c r="G13" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H13" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>37</v>
       </c>
@@ -768,8 +827,11 @@
       <c r="G14" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H14" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>37</v>
       </c>
@@ -791,8 +853,11 @@
       <c r="G15" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>42</v>
       </c>
@@ -814,8 +879,11 @@
       <c r="G16" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>42</v>
       </c>
@@ -837,8 +905,11 @@
       <c r="G17" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H17" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>50</v>
       </c>
@@ -860,8 +931,11 @@
       <c r="G18" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H18" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>7</v>
       </c>
@@ -883,8 +957,11 @@
       <c r="G19" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>7</v>
       </c>
@@ -906,8 +983,11 @@
       <c r="G20" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H20" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>7</v>
       </c>
@@ -929,8 +1009,11 @@
       <c r="G21" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H21" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>17</v>
       </c>
@@ -952,8 +1035,11 @@
       <c r="G22" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H22" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>17</v>
       </c>
@@ -975,8 +1061,11 @@
       <c r="G23" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H23" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>17</v>
       </c>
@@ -998,8 +1087,11 @@
       <c r="G24" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>17</v>
       </c>
@@ -1021,8 +1113,11 @@
       <c r="G25" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H25" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>48</v>
       </c>
@@ -1044,8 +1139,11 @@
       <c r="G26" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H26" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>48</v>
       </c>
@@ -1067,8 +1165,11 @@
       <c r="G27" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H27" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>49</v>
       </c>
@@ -1090,8 +1191,11 @@
       <c r="G28" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H28" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>49</v>
       </c>
@@ -1113,8 +1217,11 @@
       <c r="G29" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H29" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>37</v>
       </c>
@@ -1136,8 +1243,11 @@
       <c r="G30" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H30" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>37</v>
       </c>
@@ -1159,8 +1269,11 @@
       <c r="G31" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H31" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>37</v>
       </c>
@@ -1182,8 +1295,11 @@
       <c r="G32" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H32" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>42</v>
       </c>
@@ -1205,10 +1321,13 @@
       <c r="G33" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H33" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B34" t="s">
         <v>51</v>
@@ -1228,10 +1347,13 @@
       <c r="G34" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H34" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B35" t="s">
         <v>51</v>
@@ -1251,10 +1373,13 @@
       <c r="G35" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H35" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B36" t="s">
         <v>14</v>
@@ -1274,10 +1399,13 @@
       <c r="G36" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H36" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B37" t="s">
         <v>18</v>
@@ -1297,10 +1425,13 @@
       <c r="G37" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H37" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B38" t="s">
         <v>18</v>
@@ -1320,10 +1451,13 @@
       <c r="G38" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="H38" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B39" t="s">
         <v>56</v>
@@ -1334,114 +1468,129 @@
       <c r="D39" t="s">
         <v>22</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="E39" s="1">
+        <v>98496</v>
+      </c>
+      <c r="F39" t="s">
         <v>57</v>
-      </c>
-      <c r="F39" t="s">
-        <v>58</v>
       </c>
       <c r="G39" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H39" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="B40" t="s">
-        <v>14</v>
+        <v>56</v>
       </c>
       <c r="C40" t="s">
         <v>9</v>
       </c>
       <c r="D40" t="s">
-        <v>15</v>
-      </c>
-      <c r="E40">
-        <v>98493</v>
+        <v>22</v>
+      </c>
+      <c r="E40" s="1">
+        <v>98472</v>
       </c>
       <c r="F40" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
       <c r="G40" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A41" s="2" t="s">
+      <c r="H40" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>48</v>
       </c>
       <c r="B41" t="s">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="C41" t="s">
         <v>9</v>
       </c>
       <c r="D41" t="s">
-        <v>60</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>61</v>
+        <v>15</v>
+      </c>
+      <c r="E41">
+        <v>98493</v>
       </c>
       <c r="F41" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="G41" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+      <c r="H41" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
         <v>48</v>
       </c>
       <c r="B42" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C42" t="s">
         <v>9</v>
       </c>
       <c r="D42" t="s">
-        <v>24</v>
-      </c>
-      <c r="E42">
-        <v>98470</v>
+        <v>59</v>
+      </c>
+      <c r="E42" s="1">
+        <v>98503</v>
       </c>
       <c r="F42" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="G42" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+      <c r="H42" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
         <v>48</v>
       </c>
       <c r="B43" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="C43" t="s">
         <v>9</v>
       </c>
       <c r="D43" t="s">
-        <v>33</v>
-      </c>
-      <c r="E43">
-        <v>98471</v>
+        <v>59</v>
+      </c>
+      <c r="E43" s="1">
+        <v>98504</v>
       </c>
       <c r="F43" t="s">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="G43" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H43" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B44" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C44" t="s">
         <v>9</v>
@@ -1458,19 +1607,22 @@
       <c r="G44" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H44" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B45" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C45" t="s">
         <v>9</v>
       </c>
       <c r="D45" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E45">
         <v>98471</v>
@@ -1481,418 +1633,579 @@
       <c r="G45" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H45" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>49</v>
       </c>
       <c r="B46" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C46" t="s">
         <v>9</v>
       </c>
       <c r="D46" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E46">
-        <v>98496</v>
+        <v>98470</v>
       </c>
       <c r="F46" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="G46" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H46" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>49</v>
       </c>
       <c r="B47" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="C47" t="s">
         <v>9</v>
       </c>
       <c r="D47" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E47">
-        <v>98505</v>
+        <v>98471</v>
       </c>
       <c r="F47" t="s">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="G47" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H47" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="B48" t="s">
-        <v>14</v>
+        <v>61</v>
       </c>
       <c r="C48" t="s">
         <v>9</v>
       </c>
       <c r="D48" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E48">
-        <v>98512</v>
+        <v>98496</v>
       </c>
       <c r="F48" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G48" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H48" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="B49" t="s">
+        <v>14</v>
+      </c>
+      <c r="C49" t="s">
+        <v>9</v>
+      </c>
+      <c r="D49" t="s">
+        <v>15</v>
+      </c>
+      <c r="E49">
+        <v>98505</v>
+      </c>
+      <c r="F49" t="s">
         <v>63</v>
-      </c>
-      <c r="C49" t="s">
-        <v>9</v>
-      </c>
-      <c r="D49" t="s">
-        <v>27</v>
-      </c>
-      <c r="E49">
-        <v>98496</v>
-      </c>
-      <c r="F49" t="s">
-        <v>64</v>
       </c>
       <c r="G49" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H49" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>37</v>
       </c>
       <c r="B50" t="s">
-        <v>66</v>
+        <v>14</v>
       </c>
       <c r="C50" t="s">
         <v>9</v>
       </c>
       <c r="D50" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="E50">
-        <v>98473</v>
+        <v>98512</v>
       </c>
       <c r="F50" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="G50" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H50" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>37</v>
+      </c>
+      <c r="B51" t="s">
+        <v>61</v>
+      </c>
+      <c r="C51" t="s">
+        <v>9</v>
+      </c>
+      <c r="D51" t="s">
+        <v>27</v>
+      </c>
+      <c r="E51">
+        <v>98496</v>
+      </c>
+      <c r="F51" t="s">
+        <v>62</v>
+      </c>
+      <c r="G51" t="s">
+        <v>46</v>
+      </c>
+      <c r="H51" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>37</v>
+      </c>
+      <c r="B52" t="s">
+        <v>64</v>
+      </c>
+      <c r="C52" t="s">
+        <v>9</v>
+      </c>
+      <c r="D52" t="s">
+        <v>24</v>
+      </c>
+      <c r="E52">
+        <v>98473</v>
+      </c>
+      <c r="F52" t="s">
+        <v>57</v>
+      </c>
+      <c r="G52" t="s">
+        <v>46</v>
+      </c>
+      <c r="H52" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>66</v>
+      </c>
+      <c r="B53" t="s">
+        <v>14</v>
+      </c>
+      <c r="C53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D53" t="s">
+        <v>52</v>
+      </c>
+      <c r="E53">
+        <v>98464</v>
+      </c>
+      <c r="F53" t="s">
+        <v>53</v>
+      </c>
+      <c r="G53" t="s">
         <v>68</v>
       </c>
-      <c r="B51" t="s">
+      <c r="H53" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>66</v>
+      </c>
+      <c r="B54" t="s">
+        <v>18</v>
+      </c>
+      <c r="C54" t="s">
+        <v>9</v>
+      </c>
+      <c r="D54" t="s">
+        <v>19</v>
+      </c>
+      <c r="E54">
+        <v>98470</v>
+      </c>
+      <c r="F54" t="s">
+        <v>29</v>
+      </c>
+      <c r="G54" t="s">
+        <v>68</v>
+      </c>
+      <c r="H54" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>66</v>
+      </c>
+      <c r="B55" t="s">
+        <v>18</v>
+      </c>
+      <c r="C55" t="s">
+        <v>9</v>
+      </c>
+      <c r="D55" t="s">
+        <v>54</v>
+      </c>
+      <c r="E55">
+        <v>98471</v>
+      </c>
+      <c r="F55" t="s">
+        <v>55</v>
+      </c>
+      <c r="G55" t="s">
+        <v>68</v>
+      </c>
+      <c r="H55" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>66</v>
+      </c>
+      <c r="B56" t="s">
+        <v>56</v>
+      </c>
+      <c r="C56" t="s">
+        <v>9</v>
+      </c>
+      <c r="D56" t="s">
+        <v>22</v>
+      </c>
+      <c r="E56" s="1">
+        <v>98496</v>
+      </c>
+      <c r="F56" t="s">
+        <v>57</v>
+      </c>
+      <c r="G56" t="s">
+        <v>68</v>
+      </c>
+      <c r="H56" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>66</v>
+      </c>
+      <c r="B57" t="s">
+        <v>56</v>
+      </c>
+      <c r="C57" t="s">
+        <v>9</v>
+      </c>
+      <c r="D57" t="s">
+        <v>22</v>
+      </c>
+      <c r="E57" s="1">
+        <v>98472</v>
+      </c>
+      <c r="F57" t="s">
+        <v>57</v>
+      </c>
+      <c r="G57" t="s">
+        <v>68</v>
+      </c>
+      <c r="H57" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>48</v>
+      </c>
+      <c r="B58" t="s">
         <v>14</v>
       </c>
-      <c r="C51" t="s">
-        <v>9</v>
-      </c>
-      <c r="D51" t="s">
-        <v>52</v>
-      </c>
-      <c r="E51">
-        <v>98464</v>
-      </c>
-      <c r="F51" t="s">
-        <v>53</v>
-      </c>
-      <c r="G51" t="s">
+      <c r="C58" t="s">
+        <v>9</v>
+      </c>
+      <c r="D58" t="s">
+        <v>15</v>
+      </c>
+      <c r="E58">
+        <v>98493</v>
+      </c>
+      <c r="F58" t="s">
+        <v>16</v>
+      </c>
+      <c r="G58" t="s">
+        <v>68</v>
+      </c>
+      <c r="H58" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B59" t="s">
+        <v>58</v>
+      </c>
+      <c r="C59" t="s">
+        <v>9</v>
+      </c>
+      <c r="D59" t="s">
+        <v>59</v>
+      </c>
+      <c r="E59" s="1">
+        <v>98503</v>
+      </c>
+      <c r="F59" t="s">
+        <v>57</v>
+      </c>
+      <c r="G59" t="s">
+        <v>46</v>
+      </c>
+      <c r="H59" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B60" t="s">
+        <v>58</v>
+      </c>
+      <c r="C60" t="s">
+        <v>9</v>
+      </c>
+      <c r="D60" t="s">
+        <v>59</v>
+      </c>
+      <c r="E60" s="1">
+        <v>98504</v>
+      </c>
+      <c r="F60" t="s">
+        <v>57</v>
+      </c>
+      <c r="G60" t="s">
+        <v>46</v>
+      </c>
+      <c r="H60" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>37</v>
+      </c>
+      <c r="B61" t="s">
+        <v>14</v>
+      </c>
+      <c r="C61" t="s">
+        <v>9</v>
+      </c>
+      <c r="D61" t="s">
+        <v>15</v>
+      </c>
+      <c r="E61">
+        <v>98512</v>
+      </c>
+      <c r="F61" t="s">
+        <v>63</v>
+      </c>
+      <c r="G61" t="s">
+        <v>68</v>
+      </c>
+      <c r="H61" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>37</v>
+      </c>
+      <c r="B62" t="s">
+        <v>61</v>
+      </c>
+      <c r="C62" t="s">
+        <v>9</v>
+      </c>
+      <c r="D62" t="s">
+        <v>27</v>
+      </c>
+      <c r="E62">
+        <v>98496</v>
+      </c>
+      <c r="F62" t="s">
+        <v>62</v>
+      </c>
+      <c r="G62" t="s">
+        <v>68</v>
+      </c>
+      <c r="H62" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>37</v>
+      </c>
+      <c r="B63" t="s">
+        <v>64</v>
+      </c>
+      <c r="C63" t="s">
+        <v>9</v>
+      </c>
+      <c r="D63" t="s">
+        <v>24</v>
+      </c>
+      <c r="E63">
+        <v>98473</v>
+      </c>
+      <c r="F63" t="s">
+        <v>57</v>
+      </c>
+      <c r="G63" t="s">
+        <v>68</v>
+      </c>
+      <c r="H63" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>7</v>
+      </c>
+      <c r="B64" t="s">
+        <v>69</v>
+      </c>
+      <c r="C64" t="s">
+        <v>9</v>
+      </c>
+      <c r="D64" t="s">
+        <v>33</v>
+      </c>
+      <c r="E64">
+        <v>98473</v>
+      </c>
+      <c r="F64" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>68</v>
-      </c>
-      <c r="B52" t="s">
-        <v>18</v>
-      </c>
-      <c r="C52" t="s">
-        <v>9</v>
-      </c>
-      <c r="D52" t="s">
-        <v>19</v>
-      </c>
-      <c r="E52">
-        <v>98470</v>
-      </c>
-      <c r="F52" t="s">
-        <v>29</v>
-      </c>
-      <c r="G52" t="s">
+      <c r="G64" t="s">
+        <v>71</v>
+      </c>
+      <c r="H64" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>66</v>
+      </c>
+      <c r="B65" t="s">
+        <v>69</v>
+      </c>
+      <c r="C65" t="s">
+        <v>9</v>
+      </c>
+      <c r="D65" t="s">
+        <v>33</v>
+      </c>
+      <c r="E65">
+        <v>98473</v>
+      </c>
+      <c r="F65" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>68</v>
-      </c>
-      <c r="B53" t="s">
-        <v>18</v>
-      </c>
-      <c r="C53" t="s">
-        <v>9</v>
-      </c>
-      <c r="D53" t="s">
-        <v>54</v>
-      </c>
-      <c r="E53">
-        <v>98471</v>
-      </c>
-      <c r="F53" t="s">
-        <v>55</v>
-      </c>
-      <c r="G53" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>68</v>
-      </c>
-      <c r="B54" t="s">
-        <v>56</v>
-      </c>
-      <c r="C54" t="s">
-        <v>9</v>
-      </c>
-      <c r="D54" t="s">
-        <v>22</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F54" t="s">
-        <v>58</v>
-      </c>
-      <c r="G54" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>48</v>
-      </c>
-      <c r="B55" t="s">
-        <v>14</v>
-      </c>
-      <c r="C55" t="s">
-        <v>9</v>
-      </c>
-      <c r="D55" t="s">
-        <v>15</v>
-      </c>
-      <c r="E55">
-        <v>98493</v>
-      </c>
-      <c r="F55" t="s">
-        <v>16</v>
-      </c>
-      <c r="G55" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A56" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B56" t="s">
-        <v>59</v>
-      </c>
-      <c r="C56" t="s">
-        <v>9</v>
-      </c>
-      <c r="D56" t="s">
-        <v>60</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="F56" t="s">
-        <v>58</v>
-      </c>
-      <c r="G56" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>37</v>
-      </c>
-      <c r="B57" t="s">
-        <v>14</v>
-      </c>
-      <c r="C57" t="s">
-        <v>9</v>
-      </c>
-      <c r="D57" t="s">
-        <v>15</v>
-      </c>
-      <c r="E57">
-        <v>98512</v>
-      </c>
-      <c r="F57" t="s">
-        <v>65</v>
-      </c>
-      <c r="G57" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>37</v>
-      </c>
-      <c r="B58" t="s">
-        <v>63</v>
-      </c>
-      <c r="C58" t="s">
-        <v>9</v>
-      </c>
-      <c r="D58" t="s">
-        <v>27</v>
-      </c>
-      <c r="E58">
-        <v>98496</v>
-      </c>
-      <c r="F58" t="s">
-        <v>64</v>
-      </c>
-      <c r="G58" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>37</v>
-      </c>
-      <c r="B59" t="s">
-        <v>66</v>
-      </c>
-      <c r="C59" t="s">
-        <v>9</v>
-      </c>
-      <c r="D59" t="s">
-        <v>24</v>
-      </c>
-      <c r="E59">
-        <v>98473</v>
-      </c>
-      <c r="F59" t="s">
-        <v>58</v>
-      </c>
-      <c r="G59" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+      <c r="G65" t="s">
+        <v>71</v>
+      </c>
+      <c r="H65" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
         <v>7</v>
       </c>
-      <c r="B60" t="s">
-        <v>71</v>
-      </c>
-      <c r="C60" t="s">
-        <v>9</v>
-      </c>
-      <c r="D60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E60">
-        <v>98473</v>
-      </c>
-      <c r="F60" t="s">
+      <c r="B66" t="s">
         <v>72</v>
       </c>
-      <c r="G60" t="s">
+      <c r="C66" t="s">
+        <v>9</v>
+      </c>
+      <c r="D66" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>68</v>
-      </c>
-      <c r="B61" t="s">
-        <v>71</v>
-      </c>
-      <c r="C61" t="s">
-        <v>9</v>
-      </c>
-      <c r="D61" t="s">
-        <v>33</v>
-      </c>
-      <c r="E61">
-        <v>98473</v>
-      </c>
-      <c r="F61" t="s">
+      <c r="E66">
+        <v>98525</v>
+      </c>
+      <c r="F66" t="s">
+        <v>13</v>
+      </c>
+      <c r="G66" t="s">
+        <v>74</v>
+      </c>
+      <c r="H66" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>17</v>
+      </c>
+      <c r="B67" t="s">
         <v>72</v>
       </c>
-      <c r="G61" t="s">
+      <c r="C67" t="s">
+        <v>9</v>
+      </c>
+      <c r="D67" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>7</v>
-      </c>
-      <c r="B62" t="s">
+      <c r="E67">
+        <v>98525</v>
+      </c>
+      <c r="F67" t="s">
+        <v>13</v>
+      </c>
+      <c r="G67" t="s">
         <v>74</v>
       </c>
-      <c r="C62" t="s">
-        <v>9</v>
-      </c>
-      <c r="D62" t="s">
-        <v>75</v>
-      </c>
-      <c r="E62">
-        <v>98525</v>
-      </c>
-      <c r="F62" t="s">
-        <v>13</v>
-      </c>
-      <c r="G62" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>17</v>
-      </c>
-      <c r="B63" t="s">
-        <v>74</v>
-      </c>
-      <c r="C63" t="s">
-        <v>9</v>
-      </c>
-      <c r="D63" t="s">
-        <v>75</v>
-      </c>
-      <c r="E63">
-        <v>98525</v>
-      </c>
-      <c r="F63" t="s">
-        <v>13</v>
-      </c>
-      <c r="G63" t="s">
+      <c r="H67" t="s">
         <v>76</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Monday BSCS-2 classes
</commit_message>
<xml_diff>
--- a/Cleaned_Schedule/class_schedule_BSCS-4.xlsx
+++ b/Cleaned_Schedule/class_schedule_BSCS-4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neera\OneDrive\University\Spring 2025\AI\Project\Cleaned_Schedule\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCF528AE-4A13-4C88-B951-108E74139C8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1937214-7321-49A9-AE6F-7A00D5050388}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13056" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="fc898cd5-f00c-4aee-b7a7-fcde217" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="112">
   <si>
     <t>Class Timing</t>
   </si>
@@ -350,14 +350,6 @@
   </si>
   <si>
     <t>EVENT HALL</t>
-  </si>
-  <si>
-    <t>98673
-98674</t>
-  </si>
-  <si>
-    <t>Topics in History (2 Credit Hours) - (Wednesday Only from 2:30pm to 4:10pm) 
-Arabic-I (Lab Monday 2:30pm to 3:30pm)</t>
   </si>
   <si>
     <t>MAS-1</t>
@@ -556,15 +548,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H94"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.109375" customWidth="1"/>
     <col min="2" max="2" width="88.5546875" customWidth="1"/>
     <col min="3" max="3" width="8.33203125" customWidth="1"/>
-    <col min="4" max="4" width="10.21875" customWidth="1"/>
+    <col min="4" max="4" width="19.21875" customWidth="1"/>
     <col min="5" max="5" width="22.44140625" customWidth="1"/>
-    <col min="6" max="6" width="19.21875" customWidth="1"/>
+    <col min="6" max="6" width="24.88671875" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
     <col min="8" max="8" width="27.109375" customWidth="1"/>
     <col min="9" max="9" width="74.21875" customWidth="1"/>
@@ -2313,6 +2305,9 @@
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>65</v>
+      </c>
       <c r="B68" t="s">
         <v>85</v>
       </c>
@@ -2328,8 +2323,14 @@
       <c r="F68" t="s">
         <v>86</v>
       </c>
+      <c r="G68" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>65</v>
+      </c>
       <c r="B69" t="s">
         <v>87</v>
       </c>
@@ -2345,8 +2346,14 @@
       <c r="F69" t="s">
         <v>89</v>
       </c>
+      <c r="G69" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>65</v>
+      </c>
       <c r="B70" t="s">
         <v>90</v>
       </c>
@@ -2362,39 +2369,54 @@
       <c r="F70" t="s">
         <v>92</v>
       </c>
+      <c r="G70" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>66</v>
+      </c>
       <c r="B71" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C71" t="s">
         <v>84</v>
       </c>
       <c r="D71" t="s">
-        <v>54</v>
+        <v>88</v>
       </c>
       <c r="E71">
-        <v>98363</v>
+        <v>98362</v>
       </c>
       <c r="F71" t="s">
-        <v>93</v>
+        <v>95</v>
+      </c>
+      <c r="G71" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>66</v>
+      </c>
       <c r="B72" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C72" t="s">
         <v>84</v>
       </c>
       <c r="D72" t="s">
-        <v>88</v>
+        <v>54</v>
       </c>
       <c r="E72">
-        <v>98414</v>
+        <v>98363</v>
       </c>
       <c r="F72" t="s">
-        <v>95</v>
+        <v>93</v>
+      </c>
+      <c r="G72" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
@@ -2405,30 +2427,36 @@
         <v>84</v>
       </c>
       <c r="D73" t="s">
-        <v>54</v>
+        <v>88</v>
       </c>
       <c r="E73">
-        <v>98407</v>
+        <v>98414</v>
       </c>
       <c r="F73" t="s">
-        <v>93</v>
+        <v>95</v>
+      </c>
+      <c r="G73" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B74" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C74" t="s">
         <v>84</v>
       </c>
       <c r="D74" t="s">
-        <v>88</v>
+        <v>54</v>
       </c>
       <c r="E74">
-        <v>98388</v>
+        <v>98407</v>
       </c>
       <c r="F74" t="s">
-        <v>96</v>
+        <v>93</v>
+      </c>
+      <c r="G74" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
@@ -2439,149 +2467,250 @@
         <v>84</v>
       </c>
       <c r="D75" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="E75">
-        <v>98686</v>
+        <v>98388</v>
       </c>
       <c r="F75" t="s">
-        <v>98</v>
+        <v>96</v>
+      </c>
+      <c r="G75" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B76" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C76" t="s">
         <v>84</v>
       </c>
       <c r="D76" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E76">
-        <v>98868</v>
+        <v>98686</v>
       </c>
       <c r="F76" t="s">
-        <v>100</v>
+        <v>98</v>
+      </c>
+      <c r="G76" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B77" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="C77" t="s">
         <v>84</v>
       </c>
       <c r="D77" t="s">
-        <v>102</v>
-      </c>
-      <c r="E77" t="s">
-        <v>103</v>
+        <v>99</v>
+      </c>
+      <c r="E77">
+        <v>98868</v>
       </c>
       <c r="F77" t="s">
-        <v>13</v>
+        <v>100</v>
+      </c>
+      <c r="G77" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B78" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C78" t="s">
         <v>84</v>
       </c>
       <c r="D78" t="s">
-        <v>105</v>
-      </c>
-      <c r="E78" t="s">
-        <v>106</v>
+        <v>102</v>
+      </c>
+      <c r="E78" s="1">
+        <v>98673</v>
       </c>
       <c r="F78" t="s">
-        <v>107</v>
+        <v>13</v>
+      </c>
+      <c r="G78" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B79" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="C79" t="s">
         <v>84</v>
       </c>
       <c r="D79" t="s">
-        <v>97</v>
-      </c>
-      <c r="E79">
-        <v>98555</v>
+        <v>102</v>
+      </c>
+      <c r="E79" s="1">
+        <v>98674</v>
       </c>
       <c r="F79" t="s">
-        <v>98</v>
+        <v>13</v>
+      </c>
+      <c r="G79" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B80" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="C80" t="s">
         <v>84</v>
       </c>
       <c r="D80" t="s">
-        <v>102</v>
-      </c>
-      <c r="E80" t="s">
-        <v>103</v>
+        <v>97</v>
+      </c>
+      <c r="E80">
+        <v>98555</v>
       </c>
       <c r="F80" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+      <c r="G80" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="81" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B81" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C81" t="s">
         <v>84</v>
       </c>
       <c r="D81" t="s">
-        <v>105</v>
-      </c>
-      <c r="E81">
-        <v>98715</v>
+        <v>102</v>
+      </c>
+      <c r="E81" s="1">
+        <v>98673</v>
       </c>
       <c r="F81" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="G81" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="82" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B82" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="C82" t="s">
         <v>84</v>
       </c>
       <c r="D82" t="s">
-        <v>110</v>
-      </c>
-      <c r="E82">
-        <v>98444</v>
+        <v>102</v>
+      </c>
+      <c r="E82" s="1">
+        <v>98674</v>
       </c>
       <c r="F82" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="G82" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="83" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B83" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C83" t="s">
         <v>84</v>
       </c>
       <c r="D83" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="E83">
+        <v>98715</v>
+      </c>
+      <c r="F83" t="s">
+        <v>105</v>
+      </c>
+      <c r="G83" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="84" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B84" t="s">
+        <v>107</v>
+      </c>
+      <c r="C84" t="s">
+        <v>84</v>
+      </c>
+      <c r="D84" t="s">
+        <v>108</v>
+      </c>
+      <c r="E84">
+        <v>98444</v>
+      </c>
+      <c r="F84" t="s">
+        <v>109</v>
+      </c>
+      <c r="G84" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="85" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B85" t="s">
+        <v>94</v>
+      </c>
+      <c r="C85" t="s">
+        <v>84</v>
+      </c>
+      <c r="D85" t="s">
+        <v>110</v>
+      </c>
+      <c r="E85">
         <v>98446</v>
       </c>
-      <c r="F83" t="s">
-        <v>113</v>
+      <c r="F85" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="93" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B93" t="s">
+        <v>106</v>
+      </c>
+      <c r="C93" t="s">
+        <v>84</v>
+      </c>
+      <c r="D93" t="s">
+        <v>103</v>
+      </c>
+      <c r="E93" t="s">
+        <v>104</v>
+      </c>
+      <c r="F93" t="s">
+        <v>105</v>
+      </c>
+      <c r="G93" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="94" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B94" t="s">
+        <v>106</v>
+      </c>
+      <c r="C94" t="s">
+        <v>84</v>
+      </c>
+      <c r="D94" t="s">
+        <v>103</v>
+      </c>
+      <c r="E94">
+        <v>98715</v>
+      </c>
+      <c r="F94" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>